<commit_message>
Add bio link scanning moderation
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rec405b38fc7848c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="Rb606e7e5b3a2412e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R82004b10c658487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Ra3e22e03925345eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="R4041153ad6db4b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R79806367de8b4ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R0b7ac32f9e844f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R7338927984f04f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R52c770f6c1e14c86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R3d1618ef548f4d7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R56d78e97fdcd408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rbd60f7ebb7fb4bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Reed3d443488c4668"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R4a32bbc4cd244ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="Rf84834f9082b4dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R06ffdf3acc954e58"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -475,66 +475,74 @@
         <x:v>remove_unknown_bots</x:v>
       </x:c>
       <x:c r="I1" s="7" t="str">
+        <x:v>scan_bio_links</x:v>
+      </x:c>
+      <x:c r="J1" s="7" t="str">
+        <x:v>bio_scan_cache_seconds</x:v>
+      </x:c>
+      <x:c r="K1" s="7" t="str">
+        <x:v>bio_link_restrict_seconds</x:v>
+      </x:c>
+      <x:c r="L1" s="7" t="str">
+        <x:v>bio_link_warning_text</x:v>
+      </x:c>
+      <x:c r="M1" s="7" t="str">
         <x:v>exempt_admins</x:v>
       </x:c>
-      <x:c r="J1" s="7" t="str">
+      <x:c r="N1" s="7" t="str">
         <x:v>spam_max_messages</x:v>
       </x:c>
-      <x:c r="K1" s="7" t="str">
+      <x:c r="O1" s="7" t="str">
         <x:v>spam_window_seconds</x:v>
       </x:c>
-      <x:c r="L1" s="7" t="str">
+      <x:c r="P1" s="7" t="str">
         <x:v>spam_action</x:v>
       </x:c>
-      <x:c r="M1" s="7" t="str">
+      <x:c r="Q1" s="7" t="str">
         <x:v>forward_action</x:v>
       </x:c>
-      <x:c r="N1" s="7" t="str">
+      <x:c r="R1" s="7" t="str">
         <x:v>inline_keyboard_action</x:v>
       </x:c>
-      <x:c r="O1" s="7" t="str">
+      <x:c r="S1" s="7" t="str">
         <x:v>ban_after_warnings</x:v>
       </x:c>
-      <x:c r="P1" s="7" t="str">
+      <x:c r="T1" s="7" t="str">
         <x:v>warning_text</x:v>
       </x:c>
-      <x:c r="Q1" s="7" t="str">
+      <x:c r="U1" s="7" t="str">
         <x:v>daily_enabled</x:v>
       </x:c>
-      <x:c r="R1" s="7" t="str">
+      <x:c r="V1" s="7" t="str">
         <x:v>daily_window_start</x:v>
       </x:c>
-      <x:c r="S1" s="7" t="str">
+      <x:c r="W1" s="7" t="str">
         <x:v>daily_window_end</x:v>
       </x:c>
-      <x:c r="T1" s="7" t="str">
+      <x:c r="X1" s="7" t="str">
         <x:v>send_if_silent</x:v>
       </x:c>
-      <x:c r="U1" s="7" t="str">
+      <x:c r="Y1" s="7" t="str">
         <x:v>message_pool</x:v>
       </x:c>
-      <x:c r="V1" s="7" t="str">
+      <x:c r="Z1" s="7" t="str">
         <x:v>video_enabled</x:v>
       </x:c>
-      <x:c r="W1" s="7" t="str">
+      <x:c r="AA1" s="7" t="str">
         <x:v>video_window_start</x:v>
       </x:c>
-      <x:c r="X1" s="7" t="str">
+      <x:c r="AB1" s="7" t="str">
         <x:v>video_window_end</x:v>
       </x:c>
-      <x:c r="Y1" s="7" t="str">
+      <x:c r="AC1" s="7" t="str">
         <x:v>video_pool</x:v>
       </x:c>
-      <x:c r="Z1" s="7" t="str">
+      <x:c r="AD1" s="7" t="str">
         <x:v>policy_text</x:v>
       </x:c>
-      <x:c r="AA1" s="7" t="str">
+      <x:c r="AE1" s="7" t="str">
         <x:v>notes</x:v>
       </x:c>
-      <x:c r="AB1" s="8"/>
-      <x:c r="AC1" s="8"/>
-      <x:c r="AD1" s="8"/>
-      <x:c r="AE1" s="8"/>
       <x:c r="AF1" s="8"/>
       <x:c r="AG1" s="8"/>
       <x:c r="AH1" s="8"/>
@@ -586,55 +594,67 @@
         <x:v>true</x:v>
       </x:c>
       <x:c r="J2" s="2" t="n">
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L2" s="2" t="str">
+        <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
+      </x:c>
+      <x:c r="M2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="N2" s="2" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="K2" s="2" t="n">
+      <x:c r="O2" s="2" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="L2" s="2" t="str">
+      <x:c r="P2" s="2" t="str">
         <x:v>warn</x:v>
       </x:c>
-      <x:c r="M2" s="2" t="str">
+      <x:c r="Q2" s="2" t="str">
         <x:v>warn</x:v>
       </x:c>
-      <x:c r="N2" s="2" t="str">
+      <x:c r="R2" s="2" t="str">
         <x:v>warn</x:v>
       </x:c>
-      <x:c r="O2" s="2" t="n">
+      <x:c r="S2" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P2" s="2" t="str">
+      <x:c r="T2" s="2" t="str">
         <x:v>Canh bao: {reason} ({count}/{limit})</x:v>
       </x:c>
-      <x:c r="Q2" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="R2" s="2" t="str">
+      <x:c r="U2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="V2" s="2" t="str">
         <x:v>20:00</x:v>
       </x:c>
-      <x:c r="S2" s="2" t="str">
+      <x:c r="W2" s="2" t="str">
         <x:v>23:59</x:v>
       </x:c>
-      <x:c r="T2" s="2" t="str">
+      <x:c r="X2" s="2" t="str">
         <x:v>false</x:v>
-      </x:c>
-      <x:c r="U2" s="2" t="str">
-        <x:v>default</x:v>
-      </x:c>
-      <x:c r="V2" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="W2" s="2" t="str">
-        <x:v>21:00</x:v>
-      </x:c>
-      <x:c r="X2" s="2" t="str">
-        <x:v>23:00</x:v>
       </x:c>
       <x:c r="Y2" s="2" t="str">
         <x:v>default</x:v>
       </x:c>
-      <x:c r="Z2" s="2" t="str"/>
+      <x:c r="Z2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
       <x:c r="AA2" s="2" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="AB2" s="2" t="str">
+        <x:v>23:00</x:v>
+      </x:c>
+      <x:c r="AC2" s="2" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="AD2" s="2" t="str"/>
+      <x:c r="AE2" s="2" t="str">
         <x:v>Doi group_id thanh group that</x:v>
       </x:c>
     </x:row>
@@ -667,55 +687,67 @@
         <x:v>true</x:v>
       </x:c>
       <x:c r="J3" s="2" t="n">
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L3" s="2" t="str">
+        <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
+      </x:c>
+      <x:c r="M3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="N3" s="2" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="K3" s="2" t="n">
+      <x:c r="O3" s="2" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="L3" s="2" t="str">
+      <x:c r="P3" s="2" t="str">
         <x:v>delete</x:v>
       </x:c>
-      <x:c r="M3" s="2" t="str">
+      <x:c r="Q3" s="2" t="str">
         <x:v>delete</x:v>
       </x:c>
-      <x:c r="N3" s="2" t="str">
+      <x:c r="R3" s="2" t="str">
         <x:v>warn</x:v>
       </x:c>
-      <x:c r="O3" s="2" t="n">
+      <x:c r="S3" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P3" s="2" t="str">
+      <x:c r="T3" s="2" t="str">
         <x:v>Canh bao: {reason} ({count}/{limit})</x:v>
       </x:c>
-      <x:c r="Q3" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="R3" s="2" t="str">
+      <x:c r="U3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="V3" s="2" t="str">
         <x:v>19:00</x:v>
       </x:c>
-      <x:c r="S3" s="2" t="str">
+      <x:c r="W3" s="2" t="str">
         <x:v>22:00</x:v>
       </x:c>
-      <x:c r="T3" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="U3" s="2" t="str">
+      <x:c r="X3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="Y3" s="2" t="str">
         <x:v>sales</x:v>
       </x:c>
-      <x:c r="V3" s="2" t="str">
+      <x:c r="Z3" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="W3" s="2" t="str">
+      <x:c r="AA3" s="2" t="str">
         <x:v>21:00</x:v>
       </x:c>
-      <x:c r="X3" s="2" t="str">
+      <x:c r="AB3" s="2" t="str">
         <x:v>23:00</x:v>
       </x:c>
-      <x:c r="Y3" s="2" t="str">
+      <x:c r="AC3" s="2" t="str">
         <x:v>default</x:v>
       </x:c>
-      <x:c r="Z3" s="2" t="str"/>
-      <x:c r="AA3" s="2" t="str">
+      <x:c r="AD3" s="2" t="str"/>
+      <x:c r="AE3" s="2" t="str">
         <x:v>Dong mau, co the xoa</x:v>
       </x:c>
     </x:row>
@@ -747,6 +779,10 @@
       <x:c r="Y4" s="2" t="str"/>
       <x:c r="Z4" s="2" t="str"/>
       <x:c r="AA4" s="2" t="str"/>
+      <x:c r="AB4" s="2" t="str"/>
+      <x:c r="AC4" s="2" t="str"/>
+      <x:c r="AD4" s="2" t="str"/>
+      <x:c r="AE4" s="2" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -885,7 +921,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str">
-        <x:v>exempt_admins</x:v>
+        <x:v>scan_bio_links</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
         <x:v>true</x:v>
@@ -896,10 +932,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>spam_max_messages</x:v>
+        <x:v>bio_scan_cache_seconds</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>6</x:v>
+        <x:v>3600</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
         <x:v>true</x:v>
@@ -907,10 +943,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
-        <x:v>spam_window_seconds</x:v>
+        <x:v>bio_link_restrict_seconds</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
         <x:v>true</x:v>
@@ -918,10 +954,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>spam_action</x:v>
+        <x:v>bio_link_warning_text</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
         <x:v>true</x:v>
@@ -929,10 +965,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="str">
-        <x:v>forward_action</x:v>
+        <x:v>exempt_admins</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
         <x:v>true</x:v>
@@ -940,10 +976,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="str">
-        <x:v>inline_keyboard_action</x:v>
+        <x:v>spam_max_messages</x:v>
       </x:c>
       <x:c r="B13" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>true</x:v>
@@ -951,10 +987,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2" t="str">
-        <x:v>ban_after_warnings</x:v>
+        <x:v>spam_window_seconds</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
         <x:v>true</x:v>
@@ -962,10 +998,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2" t="str">
-        <x:v>daily_window_start</x:v>
+        <x:v>spam_action</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>20:00</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
         <x:v>true</x:v>
@@ -973,10 +1009,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="str">
-        <x:v>daily_window_end</x:v>
+        <x:v>forward_action</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>23:59</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
         <x:v>true</x:v>
@@ -984,10 +1020,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>send_if_silent</x:v>
+        <x:v>inline_keyboard_action</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>false</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
         <x:v>true</x:v>
@@ -995,12 +1031,56 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
+        <x:v>ban_after_warnings</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="str">
+        <x:v>daily_window_start</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>20:00</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="str">
+        <x:v>daily_window_end</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>23:59</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="str">
+        <x:v>send_if_silent</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="str">
         <x:v>send_on_boot</x:v>
       </x:c>
-      <x:c r="B18" s="2" t="str">
+      <x:c r="B22" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="C18" s="2" t="str">
+      <x:c r="C22" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add group moderation diagnostics
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R52c770f6c1e14c86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R3d1618ef548f4d7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R56d78e97fdcd408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rbd60f7ebb7fb4bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Reed3d443488c4668"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R4a32bbc4cd244ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="Rf84834f9082b4dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R06ffdf3acc954e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rcf2b25979caa4a1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="Re45d4984ea334110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R9ac9107470594832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="R485adbe4071d4096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="R9498c39fbbfc4183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="Ra7e1f5a0d9c247ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="Rf003818a5e19491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="Rbfd82805211446f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -460,90 +460,92 @@
         <x:v>enabled</x:v>
       </x:c>
       <x:c r="D1" s="7" t="str">
+        <x:v>moderation_enabled</x:v>
+      </x:c>
+      <x:c r="E1" s="7" t="str">
         <x:v>delete_system_messages</x:v>
       </x:c>
-      <x:c r="E1" s="7" t="str">
+      <x:c r="F1" s="7" t="str">
         <x:v>delete_forwarded_messages</x:v>
       </x:c>
-      <x:c r="F1" s="7" t="str">
+      <x:c r="G1" s="7" t="str">
         <x:v>delete_inline_keyboard_messages</x:v>
       </x:c>
-      <x:c r="G1" s="7" t="str">
+      <x:c r="H1" s="7" t="str">
         <x:v>delete_messages_from_bots</x:v>
       </x:c>
-      <x:c r="H1" s="7" t="str">
+      <x:c r="I1" s="7" t="str">
         <x:v>remove_unknown_bots</x:v>
       </x:c>
-      <x:c r="I1" s="7" t="str">
+      <x:c r="J1" s="7" t="str">
         <x:v>scan_bio_links</x:v>
       </x:c>
-      <x:c r="J1" s="7" t="str">
+      <x:c r="K1" s="7" t="str">
         <x:v>bio_scan_cache_seconds</x:v>
       </x:c>
-      <x:c r="K1" s="7" t="str">
+      <x:c r="L1" s="7" t="str">
         <x:v>bio_link_restrict_seconds</x:v>
       </x:c>
-      <x:c r="L1" s="7" t="str">
+      <x:c r="M1" s="7" t="str">
         <x:v>bio_link_warning_text</x:v>
       </x:c>
-      <x:c r="M1" s="7" t="str">
+      <x:c r="N1" s="7" t="str">
         <x:v>exempt_admins</x:v>
       </x:c>
-      <x:c r="N1" s="7" t="str">
+      <x:c r="O1" s="7" t="str">
         <x:v>spam_max_messages</x:v>
       </x:c>
-      <x:c r="O1" s="7" t="str">
+      <x:c r="P1" s="7" t="str">
         <x:v>spam_window_seconds</x:v>
       </x:c>
-      <x:c r="P1" s="7" t="str">
+      <x:c r="Q1" s="7" t="str">
         <x:v>spam_action</x:v>
       </x:c>
-      <x:c r="Q1" s="7" t="str">
+      <x:c r="R1" s="7" t="str">
         <x:v>forward_action</x:v>
       </x:c>
-      <x:c r="R1" s="7" t="str">
+      <x:c r="S1" s="7" t="str">
         <x:v>inline_keyboard_action</x:v>
       </x:c>
-      <x:c r="S1" s="7" t="str">
+      <x:c r="T1" s="7" t="str">
         <x:v>ban_after_warnings</x:v>
       </x:c>
-      <x:c r="T1" s="7" t="str">
+      <x:c r="U1" s="7" t="str">
         <x:v>warning_text</x:v>
       </x:c>
-      <x:c r="U1" s="7" t="str">
+      <x:c r="V1" s="7" t="str">
         <x:v>daily_enabled</x:v>
       </x:c>
-      <x:c r="V1" s="7" t="str">
+      <x:c r="W1" s="7" t="str">
         <x:v>daily_window_start</x:v>
       </x:c>
-      <x:c r="W1" s="7" t="str">
+      <x:c r="X1" s="7" t="str">
         <x:v>daily_window_end</x:v>
       </x:c>
-      <x:c r="X1" s="7" t="str">
+      <x:c r="Y1" s="7" t="str">
         <x:v>send_if_silent</x:v>
       </x:c>
-      <x:c r="Y1" s="7" t="str">
+      <x:c r="Z1" s="7" t="str">
         <x:v>message_pool</x:v>
       </x:c>
-      <x:c r="Z1" s="7" t="str">
+      <x:c r="AA1" s="7" t="str">
         <x:v>video_enabled</x:v>
       </x:c>
-      <x:c r="AA1" s="7" t="str">
+      <x:c r="AB1" s="7" t="str">
         <x:v>video_window_start</x:v>
       </x:c>
-      <x:c r="AB1" s="7" t="str">
+      <x:c r="AC1" s="7" t="str">
         <x:v>video_window_end</x:v>
       </x:c>
-      <x:c r="AC1" s="7" t="str">
+      <x:c r="AD1" s="7" t="str">
         <x:v>video_pool</x:v>
       </x:c>
-      <x:c r="AD1" s="7" t="str">
+      <x:c r="AE1" s="7" t="str">
         <x:v>policy_text</x:v>
       </x:c>
-      <x:c r="AE1" s="7" t="str">
+      <x:c r="AF1" s="7" t="str">
         <x:v>notes</x:v>
       </x:c>
-      <x:c r="AF1" s="8"/>
       <x:c r="AG1" s="8"/>
       <x:c r="AH1" s="8"/>
       <x:c r="AI1" s="8"/>
@@ -593,26 +595,26 @@
       <x:c r="I2" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="J2" s="2" t="n">
+      <x:c r="J2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="n">
         <x:v>3600</x:v>
       </x:c>
-      <x:c r="K2" s="2" t="n">
+      <x:c r="L2" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L2" s="2" t="str">
+      <x:c r="M2" s="2" t="str">
         <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
       </x:c>
-      <x:c r="M2" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="N2" s="2" t="n">
+      <x:c r="N2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="O2" s="2" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="O2" s="2" t="n">
+      <x:c r="P2" s="2" t="n">
         <x:v>12</x:v>
-      </x:c>
-      <x:c r="P2" s="2" t="str">
-        <x:v>warn</x:v>
       </x:c>
       <x:c r="Q2" s="2" t="str">
         <x:v>warn</x:v>
@@ -620,41 +622,44 @@
       <x:c r="R2" s="2" t="str">
         <x:v>warn</x:v>
       </x:c>
-      <x:c r="S2" s="2" t="n">
+      <x:c r="S2" s="2" t="str">
+        <x:v>warn</x:v>
+      </x:c>
+      <x:c r="T2" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="T2" s="2" t="str">
+      <x:c r="U2" s="2" t="str">
         <x:v>Canh bao: {reason} ({count}/{limit})</x:v>
       </x:c>
-      <x:c r="U2" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
       <x:c r="V2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="W2" s="2" t="str">
         <x:v>20:00</x:v>
       </x:c>
-      <x:c r="W2" s="2" t="str">
+      <x:c r="X2" s="2" t="str">
         <x:v>23:59</x:v>
       </x:c>
-      <x:c r="X2" s="2" t="str">
+      <x:c r="Y2" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="Y2" s="2" t="str">
+      <x:c r="Z2" s="2" t="str">
         <x:v>default</x:v>
       </x:c>
-      <x:c r="Z2" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
       <x:c r="AA2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="AB2" s="2" t="str">
         <x:v>21:00</x:v>
       </x:c>
-      <x:c r="AB2" s="2" t="str">
+      <x:c r="AC2" s="2" t="str">
         <x:v>23:00</x:v>
       </x:c>
-      <x:c r="AC2" s="2" t="str">
+      <x:c r="AD2" s="2" t="str">
         <x:v>default</x:v>
       </x:c>
-      <x:c r="AD2" s="2" t="str"/>
-      <x:c r="AE2" s="2" t="str">
+      <x:c r="AE2" s="2" t="str"/>
+      <x:c r="AF2" s="2" t="str">
         <x:v>Doi group_id thanh group that</x:v>
       </x:c>
     </x:row>
@@ -686,68 +691,71 @@
       <x:c r="I3" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="J3" s="2" t="n">
+      <x:c r="J3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="n">
         <x:v>3600</x:v>
       </x:c>
-      <x:c r="K3" s="2" t="n">
+      <x:c r="L3" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L3" s="2" t="str">
+      <x:c r="M3" s="2" t="str">
         <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
       </x:c>
-      <x:c r="M3" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="N3" s="2" t="n">
+      <x:c r="N3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="O3" s="2" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="O3" s="2" t="n">
+      <x:c r="P3" s="2" t="n">
         <x:v>15</x:v>
-      </x:c>
-      <x:c r="P3" s="2" t="str">
-        <x:v>delete</x:v>
       </x:c>
       <x:c r="Q3" s="2" t="str">
         <x:v>delete</x:v>
       </x:c>
       <x:c r="R3" s="2" t="str">
+        <x:v>delete</x:v>
+      </x:c>
+      <x:c r="S3" s="2" t="str">
         <x:v>warn</x:v>
       </x:c>
-      <x:c r="S3" s="2" t="n">
+      <x:c r="T3" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="T3" s="2" t="str">
+      <x:c r="U3" s="2" t="str">
         <x:v>Canh bao: {reason} ({count}/{limit})</x:v>
       </x:c>
-      <x:c r="U3" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
       <x:c r="V3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="W3" s="2" t="str">
         <x:v>19:00</x:v>
       </x:c>
-      <x:c r="W3" s="2" t="str">
+      <x:c r="X3" s="2" t="str">
         <x:v>22:00</x:v>
       </x:c>
-      <x:c r="X3" s="2" t="str">
-        <x:v>true</x:v>
-      </x:c>
       <x:c r="Y3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="Z3" s="2" t="str">
         <x:v>sales</x:v>
       </x:c>
-      <x:c r="Z3" s="2" t="str">
+      <x:c r="AA3" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="AA3" s="2" t="str">
+      <x:c r="AB3" s="2" t="str">
         <x:v>21:00</x:v>
       </x:c>
-      <x:c r="AB3" s="2" t="str">
+      <x:c r="AC3" s="2" t="str">
         <x:v>23:00</x:v>
       </x:c>
-      <x:c r="AC3" s="2" t="str">
+      <x:c r="AD3" s="2" t="str">
         <x:v>default</x:v>
       </x:c>
-      <x:c r="AD3" s="2" t="str"/>
-      <x:c r="AE3" s="2" t="str">
+      <x:c r="AE3" s="2" t="str"/>
+      <x:c r="AF3" s="2" t="str">
         <x:v>Dong mau, co the xoa</x:v>
       </x:c>
     </x:row>
@@ -783,6 +791,7 @@
       <x:c r="AC4" s="2" t="str"/>
       <x:c r="AD4" s="2" t="str"/>
       <x:c r="AE4" s="2" t="str"/>
+      <x:c r="AF4" s="2" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Improve mentions and sticker spam moderation
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rcf2b25979caa4a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="Re45d4984ea334110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R9ac9107470594832"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="R485adbe4071d4096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="R9498c39fbbfc4183"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="Ra7e1f5a0d9c247ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="Rf003818a5e19491d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="Rbfd82805211446f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5de649be17a54d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R36bc2847e2c742cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R645da478532f4aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="R4c0a2997a1044bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rb675bb0b5bde43a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="Rc17d2aa9bda0474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R6bf00fd19d69486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="Rb8250f8f3c834278"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1018,10 +1018,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="str">
-        <x:v>forward_action</x:v>
+        <x:v>media_spam_max_messages</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
         <x:v>true</x:v>
@@ -1029,10 +1029,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>inline_keyboard_action</x:v>
+        <x:v>media_spam_window_seconds</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
         <x:v>true</x:v>
@@ -1040,10 +1040,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
-        <x:v>ban_after_warnings</x:v>
+        <x:v>media_spam_action</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>restrict</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>true</x:v>
@@ -1051,10 +1051,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="str">
-        <x:v>daily_window_start</x:v>
+        <x:v>spam_restrict_seconds</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>20:00</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
         <x:v>true</x:v>
@@ -1062,10 +1062,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="str">
-        <x:v>daily_window_end</x:v>
+        <x:v>bio_link_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>23:59</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
         <x:v>true</x:v>
@@ -1073,10 +1073,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>send_if_silent</x:v>
+        <x:v>spam_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>false</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
         <x:v>true</x:v>
@@ -1084,12 +1084,78 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
+        <x:v>forward_action</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>warn</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="str">
+        <x:v>inline_keyboard_action</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>warn</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="str">
+        <x:v>ban_after_warnings</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="str">
+        <x:v>daily_window_start</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>20:00</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="str">
+        <x:v>daily_window_end</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>23:59</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="str">
+        <x:v>send_if_silent</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="str">
         <x:v>send_on_boot</x:v>
       </x:c>
-      <x:c r="B22" s="2" t="str">
+      <x:c r="B28" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="C22" s="2" t="str">
+      <x:c r="C28" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add tagged warning text for forwarded posts
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5de649be17a54d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R36bc2847e2c742cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R645da478532f4aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="R4c0a2997a1044bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rb675bb0b5bde43a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="Rc17d2aa9bda0474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R6bf00fd19d69486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="Rb8250f8f3c834278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R79781f7d082e480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="Ra75fd4d6f6434bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R0f849ac667714cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rd30fd1cf5839466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rf97da9aad1184a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R01c1f0139a8a40cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="Ra6cbabd9bfe14a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R10655a7be6764599"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1018,10 +1018,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="str">
-        <x:v>media_spam_max_messages</x:v>
+        <x:v>forward_warning_reason</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>Không được forward video/bài vào nhóm.</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
         <x:v>true</x:v>
@@ -1029,10 +1029,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>media_spam_window_seconds</x:v>
+        <x:v>forward_warning_text</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>10</x:v>
+        <x:v>{mention} vui lòng không forward video/bài vào nhóm. ({count}/{limit})</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
         <x:v>true</x:v>
@@ -1040,10 +1040,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
-        <x:v>media_spam_action</x:v>
+        <x:v>media_spam_max_messages</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>restrict</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>true</x:v>
@@ -1051,10 +1051,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="str">
-        <x:v>spam_restrict_seconds</x:v>
+        <x:v>media_spam_window_seconds</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>300</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
         <x:v>true</x:v>
@@ -1062,10 +1062,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="str">
-        <x:v>bio_link_notice_delete_seconds</x:v>
+        <x:v>media_spam_action</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>30</x:v>
+        <x:v>restrict</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
         <x:v>true</x:v>
@@ -1073,10 +1073,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>spam_notice_delete_seconds</x:v>
+        <x:v>spam_restrict_seconds</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>20</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
         <x:v>true</x:v>
@@ -1084,10 +1084,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
-        <x:v>forward_action</x:v>
+        <x:v>bio_link_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
         <x:v>true</x:v>
@@ -1095,10 +1095,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="str">
-        <x:v>inline_keyboard_action</x:v>
+        <x:v>spam_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B23" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C23" s="2" t="str">
         <x:v>true</x:v>
@@ -1106,10 +1106,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="2" t="str">
-        <x:v>ban_after_warnings</x:v>
+        <x:v>forward_action</x:v>
       </x:c>
       <x:c r="B24" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C24" s="2" t="str">
         <x:v>true</x:v>
@@ -1117,10 +1117,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="2" t="str">
-        <x:v>daily_window_start</x:v>
+        <x:v>inline_keyboard_action</x:v>
       </x:c>
       <x:c r="B25" s="2" t="str">
-        <x:v>20:00</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C25" s="2" t="str">
         <x:v>true</x:v>
@@ -1128,10 +1128,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="2" t="str">
-        <x:v>daily_window_end</x:v>
+        <x:v>ban_after_warnings</x:v>
       </x:c>
       <x:c r="B26" s="2" t="str">
-        <x:v>23:59</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
         <x:v>true</x:v>
@@ -1139,10 +1139,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="2" t="str">
-        <x:v>send_if_silent</x:v>
+        <x:v>daily_window_start</x:v>
       </x:c>
       <x:c r="B27" s="2" t="str">
-        <x:v>false</x:v>
+        <x:v>20:00</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
         <x:v>true</x:v>
@@ -1150,12 +1150,34 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="2" t="str">
+        <x:v>daily_window_end</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>23:59</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="str">
+        <x:v>send_if_silent</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2" t="str">
         <x:v>send_on_boot</x:v>
       </x:c>
-      <x:c r="B28" s="2" t="str">
+      <x:c r="B30" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="C28" s="2" t="str">
+      <x:c r="C30" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Auto-delete all moderation warnings
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R79781f7d082e480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="Ra75fd4d6f6434bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R0f849ac667714cc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rd30fd1cf5839466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rf97da9aad1184a43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R01c1f0139a8a40cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="Ra6cbabd9bfe14a65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R10655a7be6764599"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R13f0b056d9934535"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R8c2c400ed8714a26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R72bfdd948ea04bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rbf221dbe911b484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rb26cfb98613e4164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R2420a93e48c24499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R92dac05744ba4cd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="Rabbf1e28e487480e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1040,10 +1040,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
-        <x:v>media_spam_max_messages</x:v>
+        <x:v>forward_warning_delete_seconds</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>true</x:v>
@@ -1051,10 +1051,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="str">
-        <x:v>media_spam_window_seconds</x:v>
+        <x:v>warning_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>10</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
         <x:v>true</x:v>
@@ -1062,10 +1062,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="str">
-        <x:v>media_spam_action</x:v>
+        <x:v>media_spam_max_messages</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>restrict</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
         <x:v>true</x:v>
@@ -1073,10 +1073,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>spam_restrict_seconds</x:v>
+        <x:v>media_spam_window_seconds</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>300</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
         <x:v>true</x:v>
@@ -1084,10 +1084,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
-        <x:v>bio_link_notice_delete_seconds</x:v>
+        <x:v>media_spam_action</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>30</x:v>
+        <x:v>restrict</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
         <x:v>true</x:v>
@@ -1095,10 +1095,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="str">
-        <x:v>spam_notice_delete_seconds</x:v>
+        <x:v>spam_restrict_seconds</x:v>
       </x:c>
       <x:c r="B23" s="2" t="str">
-        <x:v>20</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C23" s="2" t="str">
         <x:v>true</x:v>
@@ -1106,10 +1106,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="2" t="str">
-        <x:v>forward_action</x:v>
+        <x:v>bio_link_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B24" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C24" s="2" t="str">
         <x:v>true</x:v>
@@ -1117,10 +1117,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="2" t="str">
-        <x:v>inline_keyboard_action</x:v>
+        <x:v>spam_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B25" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C25" s="2" t="str">
         <x:v>true</x:v>
@@ -1128,10 +1128,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="2" t="str">
-        <x:v>ban_after_warnings</x:v>
+        <x:v>forward_action</x:v>
       </x:c>
       <x:c r="B26" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
         <x:v>true</x:v>
@@ -1139,10 +1139,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="2" t="str">
-        <x:v>daily_window_start</x:v>
+        <x:v>inline_keyboard_action</x:v>
       </x:c>
       <x:c r="B27" s="2" t="str">
-        <x:v>20:00</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
         <x:v>true</x:v>
@@ -1150,10 +1150,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="2" t="str">
-        <x:v>daily_window_end</x:v>
+        <x:v>ban_after_warnings</x:v>
       </x:c>
       <x:c r="B28" s="2" t="str">
-        <x:v>23:59</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C28" s="2" t="str">
         <x:v>true</x:v>
@@ -1161,10 +1161,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="2" t="str">
-        <x:v>send_if_silent</x:v>
+        <x:v>daily_window_start</x:v>
       </x:c>
       <x:c r="B29" s="2" t="str">
-        <x:v>false</x:v>
+        <x:v>20:00</x:v>
       </x:c>
       <x:c r="C29" s="2" t="str">
         <x:v>true</x:v>
@@ -1172,12 +1172,34 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="str">
+        <x:v>daily_window_end</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>23:59</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="str">
+        <x:v>send_if_silent</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="str">
         <x:v>send_on_boot</x:v>
       </x:c>
-      <x:c r="B30" s="2" t="str">
+      <x:c r="B32" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="C30" s="2" t="str">
+      <x:c r="C32" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Ensure keyword violations are deleted before ban
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R13f0b056d9934535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R8c2c400ed8714a26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R72bfdd948ea04bfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rbf221dbe911b484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rb26cfb98613e4164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R2420a93e48c24499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R92dac05744ba4cd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="Rabbf1e28e487480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Raa95979b6ecc4f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R2f80010d488b4c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="Rc19f24991a004e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rcb29dde9e8af43be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rb2090b4e13774a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R124861c8c5ae42f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R365efde9768c4427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R6ab4912829544b32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1384,12 +1384,14 @@
         <x:v>action</x:v>
       </x:c>
       <x:c r="D1" s="7" t="str">
+        <x:v>delete</x:v>
+      </x:c>
+      <x:c r="E1" s="7" t="str">
         <x:v>reason</x:v>
       </x:c>
-      <x:c r="E1" s="7" t="str">
+      <x:c r="F1" s="7" t="str">
         <x:v>enabled</x:v>
       </x:c>
-      <x:c r="F1" s="8"/>
       <x:c r="G1" s="8"/>
       <x:c r="H1" s="8"/>
       <x:c r="I1" s="8"/>
@@ -1448,9 +1450,12 @@
         <x:v>warn</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
         <x:v>Tu khoa cam</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="str">
+      <x:c r="F2" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>
@@ -1465,9 +1470,12 @@
         <x:v>delete</x:v>
       </x:c>
       <x:c r="D3" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
         <x:v>Link spam</x:v>
       </x:c>
-      <x:c r="E3" s="2" t="str">
+      <x:c r="F3" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>
@@ -1482,9 +1490,12 @@
         <x:v>ban</x:v>
       </x:c>
       <x:c r="D4" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str">
         <x:v>Link spam nang</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="str">
+      <x:c r="F4" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>
@@ -1499,9 +1510,12 @@
         <x:v>warn</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str">
         <x:v>Noi dung spam</x:v>
       </x:c>
-      <x:c r="E5" s="2" t="str">
+      <x:c r="F5" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>
@@ -1516,9 +1530,12 @@
         <x:v>delete</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str">
         <x:v>Regex mau</x:v>
       </x:c>
-      <x:c r="E6" s="2" t="str">
+      <x:c r="F6" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
     </x:row>
@@ -1528,6 +1545,7 @@
       <x:c r="C7" s="2" t="str"/>
       <x:c r="D7" s="2" t="str"/>
       <x:c r="E7" s="2" t="str"/>
+      <x:c r="F7" s="2" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str"/>
@@ -1535,6 +1553,7 @@
       <x:c r="C8" s="2" t="str"/>
       <x:c r="D8" s="2" t="str"/>
       <x:c r="E8" s="2" t="str"/>
+      <x:c r="F8" s="2" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str"/>
@@ -1542,6 +1561,7 @@
       <x:c r="C9" s="2" t="str"/>
       <x:c r="D9" s="2" t="str"/>
       <x:c r="E9" s="2" t="str"/>
+      <x:c r="F9" s="2" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Always delete violation messages before moderation actions
</commit_message>
<xml_diff>
--- a/outputs/cu_bot_google_sheet_template.xlsx
+++ b/outputs/cu_bot_google_sheet_template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Raa95979b6ecc4f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R2f80010d488b4c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="Rc19f24991a004e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="Rcb29dde9e8af43be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rb2090b4e13774a5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R124861c8c5ae42f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R365efde9768c4427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R6ab4912829544b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7f7bcad0a7ed42f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groups" sheetId="2" r:id="R7142804944b644aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="3" r:id="R1482a83d8aa646ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="messages" sheetId="4" r:id="R5f676a377ac44014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keywords" sheetId="5" r:id="Rad6be45bc5784cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admins" sheetId="6" r:id="R519fe5aed4d04816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bot_allowlist" sheetId="7" r:id="R223ce048196d47a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="video_messages" sheetId="8" r:id="R07ccba90dfd84346"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -941,10 +941,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>bio_scan_cache_seconds</x:v>
+        <x:v>bio_link_delete_message</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>3600</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
         <x:v>true</x:v>
@@ -952,10 +952,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
-        <x:v>bio_link_restrict_seconds</x:v>
+        <x:v>bio_scan_cache_seconds</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>0</x:v>
+        <x:v>3600</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
         <x:v>true</x:v>
@@ -963,10 +963,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>bio_link_warning_text</x:v>
+        <x:v>bio_link_restrict_seconds</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
         <x:v>true</x:v>
@@ -974,10 +974,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="str">
-        <x:v>exempt_admins</x:v>
+        <x:v>bio_link_warning_text</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>true</x:v>
+        <x:v>{mention} vui long go link Telegram trong bio roi lien he admin de mo chat lai.</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
         <x:v>true</x:v>
@@ -985,10 +985,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="str">
-        <x:v>spam_max_messages</x:v>
+        <x:v>exempt_admins</x:v>
       </x:c>
       <x:c r="B13" s="2" t="str">
-        <x:v>6</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>true</x:v>
@@ -996,10 +996,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2" t="str">
-        <x:v>spam_window_seconds</x:v>
+        <x:v>spam_max_messages</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
         <x:v>true</x:v>
@@ -1007,10 +1007,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2" t="str">
-        <x:v>spam_action</x:v>
+        <x:v>spam_window_seconds</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
         <x:v>true</x:v>
@@ -1018,10 +1018,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="str">
-        <x:v>forward_warning_reason</x:v>
+        <x:v>spam_action</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>Không được forward video/bài vào nhóm.</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
         <x:v>true</x:v>
@@ -1029,10 +1029,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>forward_warning_text</x:v>
+        <x:v>forward_warning_reason</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>{mention} vui lòng không forward video/bài vào nhóm. ({count}/{limit})</x:v>
+        <x:v>Không được forward video/bài vào nhóm.</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
         <x:v>true</x:v>
@@ -1040,10 +1040,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
-        <x:v>forward_warning_delete_seconds</x:v>
+        <x:v>forward_warning_text</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>180</x:v>
+        <x:v>{mention} vui lòng không forward video/bài vào nhóm. ({count}/{limit})</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>true</x:v>
@@ -1051,7 +1051,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="str">
-        <x:v>warning_notice_delete_seconds</x:v>
+        <x:v>forward_warning_delete_seconds</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
         <x:v>180</x:v>
@@ -1062,10 +1062,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="str">
-        <x:v>media_spam_max_messages</x:v>
+        <x:v>warning_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
         <x:v>true</x:v>
@@ -1073,10 +1073,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>media_spam_window_seconds</x:v>
+        <x:v>media_spam_max_messages</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>10</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
         <x:v>true</x:v>
@@ -1084,10 +1084,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
-        <x:v>media_spam_action</x:v>
+        <x:v>media_spam_window_seconds</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>restrict</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
         <x:v>true</x:v>
@@ -1095,10 +1095,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="str">
-        <x:v>spam_restrict_seconds</x:v>
+        <x:v>media_spam_action</x:v>
       </x:c>
       <x:c r="B23" s="2" t="str">
-        <x:v>300</x:v>
+        <x:v>restrict</x:v>
       </x:c>
       <x:c r="C23" s="2" t="str">
         <x:v>true</x:v>
@@ -1106,10 +1106,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="2" t="str">
-        <x:v>bio_link_notice_delete_seconds</x:v>
+        <x:v>spam_restrict_seconds</x:v>
       </x:c>
       <x:c r="B24" s="2" t="str">
-        <x:v>30</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C24" s="2" t="str">
         <x:v>true</x:v>
@@ -1117,10 +1117,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="2" t="str">
-        <x:v>spam_notice_delete_seconds</x:v>
+        <x:v>bio_link_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B25" s="2" t="str">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C25" s="2" t="str">
         <x:v>true</x:v>
@@ -1128,10 +1128,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="2" t="str">
-        <x:v>forward_action</x:v>
+        <x:v>spam_notice_delete_seconds</x:v>
       </x:c>
       <x:c r="B26" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
         <x:v>true</x:v>
@@ -1139,10 +1139,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="2" t="str">
-        <x:v>inline_keyboard_action</x:v>
+        <x:v>violation_delete_retry_seconds</x:v>
       </x:c>
       <x:c r="B27" s="2" t="str">
-        <x:v>warn</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
         <x:v>true</x:v>
@@ -1150,10 +1150,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="2" t="str">
-        <x:v>ban_after_warnings</x:v>
+        <x:v>forward_action</x:v>
       </x:c>
       <x:c r="B28" s="2" t="str">
-        <x:v>3</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C28" s="2" t="str">
         <x:v>true</x:v>
@@ -1161,10 +1161,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="2" t="str">
-        <x:v>daily_window_start</x:v>
+        <x:v>inline_keyboard_action</x:v>
       </x:c>
       <x:c r="B29" s="2" t="str">
-        <x:v>20:00</x:v>
+        <x:v>warn</x:v>
       </x:c>
       <x:c r="C29" s="2" t="str">
         <x:v>true</x:v>
@@ -1172,10 +1172,10 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="str">
-        <x:v>daily_window_end</x:v>
+        <x:v>ban_after_warnings</x:v>
       </x:c>
       <x:c r="B30" s="2" t="str">
-        <x:v>23:59</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C30" s="2" t="str">
         <x:v>true</x:v>
@@ -1183,10 +1183,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="2" t="str">
-        <x:v>send_if_silent</x:v>
+        <x:v>daily_window_start</x:v>
       </x:c>
       <x:c r="B31" s="2" t="str">
-        <x:v>false</x:v>
+        <x:v>20:00</x:v>
       </x:c>
       <x:c r="C31" s="2" t="str">
         <x:v>true</x:v>
@@ -1194,12 +1194,34 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="2" t="str">
+        <x:v>daily_window_end</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>23:59</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="str">
+        <x:v>send_if_silent</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="str">
         <x:v>send_on_boot</x:v>
       </x:c>
-      <x:c r="B32" s="2" t="str">
+      <x:c r="B34" s="2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="C32" s="2" t="str">
+      <x:c r="C34" s="2" t="str">
         <x:v>true</x:v>
       </x:c>
     </x:row>

</xml_diff>